<commit_message>
Add trace round-trip benchmark (tracker row 9): 10 LangGraph runs through the adapter, JSON-only round-trip (model_dump_json/model_validate_json), full pass/fail reporting with a hard assert; all 10/10 passed
</commit_message>
<xml_diff>
--- a/DOCUMENTATION/project1_timeline_tracker.xlsx
+++ b/DOCUMENTATION/project1_timeline_tracker.xlsx
@@ -1,17 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\spars\Desktop\GEL\DOCUMENTATION\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C53D136-AEA9-4E90-AF66-1B0BF5EDCC90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-109" yWindow="-109" windowWidth="26301" windowHeight="14169" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Timeline Tracker" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Timeline Tracker" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -22,301 +36,299 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="95">
   <si>
-    <t xml:space="preserve">Guardrail &amp; Evaluation Layer — Build Tracker (Project 1, v3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total Tasks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% Complete</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Done</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In Progress</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Task</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Target Duration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Benchmark / Done-When</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1a — Trace Skeleton (Wk 1–4)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Design canonical trace schema</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not Started</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Build LangGraph adapter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week 1–2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Set up Postgres trace store</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Build privacy/redaction filter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week 2–3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Build provider abstraction layer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Build mock evaluator</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Implement caching layer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week 3–4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Implement retry / rate-limit handling</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Benchmark: 10 known runs round-trip, zero data loss</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zero data loss on round-trip</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Benchmark: secrets/PII confirmed redacted</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No unredacted secrets in stored traces</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Benchmark: repeated call served from cache</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Identical call not re-sent to provider</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Integration Check 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verify trace schema covers all downstream fields</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~1 day</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Every field 1b–1d needs is present</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1b — Basic Evaluation (Wk 5–6)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Build eval-signal schema (incl. evaluator_version)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week 5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Build rule-based evaluators</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Build embedding evaluators</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week 5–6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Build dataset versioning</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week 6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Create 20–30 case hand-labeled dataset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Benchmark: rule-based checks match expected pass/fail</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exact match vs. hand-labeled set</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Benchmark: embedding scores correlate with human judgment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Directional correlation confirmed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1c — Groundedness (Wk 7–9)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Build claim extraction step</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week 7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Build evidence retrieval step</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week 7–8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Build entailment check step</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week 8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Implement full metric set (claims, unsupported, contradicted, coverage, retrieval failure, extraction confidence)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week 8–9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Create labeled claim-level benchmark set</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week 9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Benchmark: entailment labels match human labels ≥ 80%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">≥80% agreement with human labels</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Integration Check 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verify groundedness results flow into eval-signal schema</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evidence + severity populated correctly</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1d — Security Suite (Wk 10–12)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Build prompt injection test module</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week 10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Build indirect injection test module</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Build permission / allow-list evaluation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week 11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Build tool-argument validation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Build loop / excessive-retry detection</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Build versioned security payload registry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week 12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Benchmark: adversarial suite catch-rate meets threshold</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Defined min. % of payloads caught</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1e — Dashboard (Wk 13–14)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Build dashboard UI skeleton</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week 13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wire eval signals with evidence &amp; severity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wire security findings view</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week 14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Benchmark: every finding traceable to trace_span_ids</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Manual walkthrough passes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Buffer (Wk 15–16)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Debugging &amp; polish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week 15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Documentation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week 15–16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Report / viva prep</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week 16</t>
+    <t>Guardrail &amp; Evaluation Layer — Build Tracker (Project 1, v3)</t>
+  </si>
+  <si>
+    <t>Total Tasks</t>
+  </si>
+  <si>
+    <t>% Complete</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>Phase</t>
+  </si>
+  <si>
+    <t>Task</t>
+  </si>
+  <si>
+    <t>Target Duration</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Benchmark / Done-When</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>1a — Trace Skeleton (Wk 1–4)</t>
+  </si>
+  <si>
+    <t>Design canonical trace schema</t>
+  </si>
+  <si>
+    <t>Week 1</t>
+  </si>
+  <si>
+    <t>Not Started</t>
+  </si>
+  <si>
+    <t>Build LangGraph adapter</t>
+  </si>
+  <si>
+    <t>Week 1–2</t>
+  </si>
+  <si>
+    <t>Set up Postgres trace store</t>
+  </si>
+  <si>
+    <t>Week 2</t>
+  </si>
+  <si>
+    <t>Build privacy/redaction filter</t>
+  </si>
+  <si>
+    <t>Week 2–3</t>
+  </si>
+  <si>
+    <t>Build provider abstraction layer</t>
+  </si>
+  <si>
+    <t>Week 3</t>
+  </si>
+  <si>
+    <t>Build mock evaluator</t>
+  </si>
+  <si>
+    <t>Implement caching layer</t>
+  </si>
+  <si>
+    <t>Week 3–4</t>
+  </si>
+  <si>
+    <t>Implement retry / rate-limit handling</t>
+  </si>
+  <si>
+    <t>Week 4</t>
+  </si>
+  <si>
+    <t>Benchmark: 10 known runs round-trip, zero data loss</t>
+  </si>
+  <si>
+    <t>Zero data loss on round-trip</t>
+  </si>
+  <si>
+    <t>Benchmark: secrets/PII confirmed redacted</t>
+  </si>
+  <si>
+    <t>No unredacted secrets in stored traces</t>
+  </si>
+  <si>
+    <t>Benchmark: repeated call served from cache</t>
+  </si>
+  <si>
+    <t>Identical call not re-sent to provider</t>
+  </si>
+  <si>
+    <t>Integration Check 1</t>
+  </si>
+  <si>
+    <t>Verify trace schema covers all downstream fields</t>
+  </si>
+  <si>
+    <t>~1 day</t>
+  </si>
+  <si>
+    <t>Every field 1b–1d needs is present</t>
+  </si>
+  <si>
+    <t>1b — Basic Evaluation (Wk 5–6)</t>
+  </si>
+  <si>
+    <t>Build eval-signal schema (incl. evaluator_version)</t>
+  </si>
+  <si>
+    <t>Week 5</t>
+  </si>
+  <si>
+    <t>Build rule-based evaluators</t>
+  </si>
+  <si>
+    <t>Build embedding evaluators</t>
+  </si>
+  <si>
+    <t>Week 5–6</t>
+  </si>
+  <si>
+    <t>Build dataset versioning</t>
+  </si>
+  <si>
+    <t>Week 6</t>
+  </si>
+  <si>
+    <t>Create 20–30 case hand-labeled dataset</t>
+  </si>
+  <si>
+    <t>Benchmark: rule-based checks match expected pass/fail</t>
+  </si>
+  <si>
+    <t>Exact match vs. hand-labeled set</t>
+  </si>
+  <si>
+    <t>Benchmark: embedding scores correlate with human judgment</t>
+  </si>
+  <si>
+    <t>Directional correlation confirmed</t>
+  </si>
+  <si>
+    <t>1c — Groundedness (Wk 7–9)</t>
+  </si>
+  <si>
+    <t>Build claim extraction step</t>
+  </si>
+  <si>
+    <t>Week 7</t>
+  </si>
+  <si>
+    <t>Build evidence retrieval step</t>
+  </si>
+  <si>
+    <t>Week 7–8</t>
+  </si>
+  <si>
+    <t>Build entailment check step</t>
+  </si>
+  <si>
+    <t>Week 8</t>
+  </si>
+  <si>
+    <t>Implement full metric set (claims, unsupported, contradicted, coverage, retrieval failure, extraction confidence)</t>
+  </si>
+  <si>
+    <t>Week 8–9</t>
+  </si>
+  <si>
+    <t>Create labeled claim-level benchmark set</t>
+  </si>
+  <si>
+    <t>Week 9</t>
+  </si>
+  <si>
+    <t>Benchmark: entailment labels match human labels ≥ 80%</t>
+  </si>
+  <si>
+    <t>≥80% agreement with human labels</t>
+  </si>
+  <si>
+    <t>Integration Check 2</t>
+  </si>
+  <si>
+    <t>Verify groundedness results flow into eval-signal schema</t>
+  </si>
+  <si>
+    <t>Evidence + severity populated correctly</t>
+  </si>
+  <si>
+    <t>1d — Security Suite (Wk 10–12)</t>
+  </si>
+  <si>
+    <t>Build prompt injection test module</t>
+  </si>
+  <si>
+    <t>Week 10</t>
+  </si>
+  <si>
+    <t>Build indirect injection test module</t>
+  </si>
+  <si>
+    <t>Build permission / allow-list evaluation</t>
+  </si>
+  <si>
+    <t>Week 11</t>
+  </si>
+  <si>
+    <t>Build tool-argument validation</t>
+  </si>
+  <si>
+    <t>Build loop / excessive-retry detection</t>
+  </si>
+  <si>
+    <t>Build versioned security payload registry</t>
+  </si>
+  <si>
+    <t>Week 12</t>
+  </si>
+  <si>
+    <t>Benchmark: adversarial suite catch-rate meets threshold</t>
+  </si>
+  <si>
+    <t>Defined min. % of payloads caught</t>
+  </si>
+  <si>
+    <t>1e — Dashboard (Wk 13–14)</t>
+  </si>
+  <si>
+    <t>Build dashboard UI skeleton</t>
+  </si>
+  <si>
+    <t>Week 13</t>
+  </si>
+  <si>
+    <t>Wire eval signals with evidence &amp; severity</t>
+  </si>
+  <si>
+    <t>Wire security findings view</t>
+  </si>
+  <si>
+    <t>Week 14</t>
+  </si>
+  <si>
+    <t>Benchmark: every finding traceable to trace_span_ids</t>
+  </si>
+  <si>
+    <t>Manual walkthrough passes</t>
+  </si>
+  <si>
+    <t>Buffer (Wk 15–16)</t>
+  </si>
+  <si>
+    <t>Debugging &amp; polish</t>
+  </si>
+  <si>
+    <t>Week 15</t>
+  </si>
+  <si>
+    <t>Documentation</t>
+  </si>
+  <si>
+    <t>Week 15–16</t>
+  </si>
+  <si>
+    <t>Report / viva prep</t>
+  </si>
+  <si>
+    <t>Week 16</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="General"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -325,55 +337,35 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
+      <b/>
       <sz val="16"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FF1F4E78"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -398,14 +390,14 @@
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left style="thin">
         <color rgb="FFB7B7B7"/>
       </left>
@@ -421,74 +413,32 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="7">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
   <dxfs count="3">
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFF2F2F2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -502,11 +452,12 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
   </dxfs>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -565,47 +516,63 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF1F4E78"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -613,12 +580,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -647,7 +614,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -668,7 +635,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -719,7 +686,7 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -737,32 +704,31 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G47"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.625" defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="24"/>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="42" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="46" customWidth="1"/>
+    <col min="7" max="7" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:7" ht="27.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -773,41 +739,41 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="n">
-        <f aca="false">COUNTA(B7:B100)-COUNTBLANK(B7:B100)</f>
+      <c r="B3" s="3">
+        <f>COUNTA(B7:B100)-COUNTBLANK(B7:B100)</f>
         <v>-12</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="4" t="n">
-        <f aca="false">IFERROR(B4/B3,0)</f>
-        <v>-0</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D3" s="4">
+        <f>IFERROR(B4/B3,0)</f>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="n">
-        <f aca="false">COUNTIF(E7:E100,"Done")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B4" s="3">
+        <f>COUNTIF(E7:E100,"Done")</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="n">
-        <f aca="false">COUNTIF(E7:E100,"In Progress")</f>
+      <c r="B5" s="3">
+        <f>COUNTIF(E7:E100,"In Progress")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:7" ht="28.55" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>5</v>
       </c>
@@ -830,8 +796,8 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="n">
+    <row r="8" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="6">
         <v>1</v>
       </c>
       <c r="B8" s="6" t="s">
@@ -844,13 +810,13 @@
         <v>14</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="F8" s="6"/>
       <c r="G8" s="6"/>
     </row>
-    <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="n">
+    <row r="9" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="6">
         <v>2</v>
       </c>
       <c r="B9" s="6" t="s">
@@ -863,13 +829,13 @@
         <v>17</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="F9" s="6"/>
       <c r="G9" s="6"/>
     </row>
-    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="n">
+    <row r="10" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="6">
         <v>3</v>
       </c>
       <c r="B10" s="6" t="s">
@@ -882,13 +848,13 @@
         <v>19</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="F10" s="6"/>
       <c r="G10" s="6"/>
     </row>
-    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="n">
+    <row r="11" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="6">
         <v>4</v>
       </c>
       <c r="B11" s="6" t="s">
@@ -901,13 +867,13 @@
         <v>21</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
     </row>
-    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="n">
+    <row r="12" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="6">
         <v>5</v>
       </c>
       <c r="B12" s="6" t="s">
@@ -920,13 +886,13 @@
         <v>23</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="F12" s="6"/>
       <c r="G12" s="6"/>
     </row>
-    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="n">
+    <row r="13" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="6">
         <v>6</v>
       </c>
       <c r="B13" s="6" t="s">
@@ -939,13 +905,13 @@
         <v>23</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="F13" s="6"/>
       <c r="G13" s="6"/>
     </row>
-    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="n">
+    <row r="14" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="6">
         <v>7</v>
       </c>
       <c r="B14" s="6" t="s">
@@ -958,13 +924,13 @@
         <v>26</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="F14" s="6"/>
       <c r="G14" s="6"/>
     </row>
-    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="n">
+    <row r="15" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="6">
         <v>8</v>
       </c>
       <c r="B15" s="6" t="s">
@@ -977,13 +943,13 @@
         <v>28</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="F15" s="6"/>
       <c r="G15" s="6"/>
     </row>
-    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="n">
+    <row r="16" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="6">
         <v>9</v>
       </c>
       <c r="B16" s="6" t="s">
@@ -996,15 +962,15 @@
         <v>28</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>30</v>
       </c>
       <c r="G16" s="6"/>
     </row>
-    <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="n">
+    <row r="17" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="6">
         <v>10</v>
       </c>
       <c r="B17" s="6" t="s">
@@ -1017,15 +983,15 @@
         <v>28</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="F17" s="6" t="s">
         <v>32</v>
       </c>
       <c r="G17" s="6"/>
     </row>
-    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="n">
+    <row r="18" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="6">
         <v>11</v>
       </c>
       <c r="B18" s="6" t="s">
@@ -1038,15 +1004,15 @@
         <v>28</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>34</v>
       </c>
       <c r="G18" s="6"/>
     </row>
-    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="n">
+    <row r="19" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="6">
         <v>12</v>
       </c>
       <c r="B19" s="6" t="s">
@@ -1059,15 +1025,15 @@
         <v>37</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="F19" s="6" t="s">
         <v>38</v>
       </c>
       <c r="G19" s="6"/>
     </row>
-    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="n">
+    <row r="20" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="6">
         <v>13</v>
       </c>
       <c r="B20" s="6" t="s">
@@ -1085,8 +1051,8 @@
       <c r="F20" s="6"/>
       <c r="G20" s="6"/>
     </row>
-    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="n">
+    <row r="21" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="6">
         <v>14</v>
       </c>
       <c r="B21" s="6" t="s">
@@ -1104,8 +1070,8 @@
       <c r="F21" s="6"/>
       <c r="G21" s="6"/>
     </row>
-    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="n">
+    <row r="22" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="6">
         <v>15</v>
       </c>
       <c r="B22" s="6" t="s">
@@ -1123,8 +1089,8 @@
       <c r="F22" s="6"/>
       <c r="G22" s="6"/>
     </row>
-    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="6" t="n">
+    <row r="23" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="6">
         <v>16</v>
       </c>
       <c r="B23" s="6" t="s">
@@ -1142,8 +1108,8 @@
       <c r="F23" s="6"/>
       <c r="G23" s="6"/>
     </row>
-    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="6" t="n">
+    <row r="24" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="6">
         <v>17</v>
       </c>
       <c r="B24" s="6" t="s">
@@ -1161,8 +1127,8 @@
       <c r="F24" s="6"/>
       <c r="G24" s="6"/>
     </row>
-    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="6" t="n">
+    <row r="25" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="6">
         <v>18</v>
       </c>
       <c r="B25" s="6" t="s">
@@ -1182,8 +1148,8 @@
       </c>
       <c r="G25" s="6"/>
     </row>
-    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="6" t="n">
+    <row r="26" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="6">
         <v>19</v>
       </c>
       <c r="B26" s="6" t="s">
@@ -1203,8 +1169,8 @@
       </c>
       <c r="G26" s="6"/>
     </row>
-    <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="6" t="n">
+    <row r="27" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="6">
         <v>20</v>
       </c>
       <c r="B27" s="6" t="s">
@@ -1222,8 +1188,8 @@
       <c r="F27" s="6"/>
       <c r="G27" s="6"/>
     </row>
-    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="6" t="n">
+    <row r="28" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="6">
         <v>21</v>
       </c>
       <c r="B28" s="6" t="s">
@@ -1241,8 +1207,8 @@
       <c r="F28" s="6"/>
       <c r="G28" s="6"/>
     </row>
-    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="6" t="n">
+    <row r="29" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="6">
         <v>22</v>
       </c>
       <c r="B29" s="6" t="s">
@@ -1260,8 +1226,8 @@
       <c r="F29" s="6"/>
       <c r="G29" s="6"/>
     </row>
-    <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="6" t="n">
+    <row r="30" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="6">
         <v>23</v>
       </c>
       <c r="B30" s="6" t="s">
@@ -1279,8 +1245,8 @@
       <c r="F30" s="6"/>
       <c r="G30" s="6"/>
     </row>
-    <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="6" t="n">
+    <row r="31" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="6">
         <v>24</v>
       </c>
       <c r="B31" s="6" t="s">
@@ -1298,8 +1264,8 @@
       <c r="F31" s="6"/>
       <c r="G31" s="6"/>
     </row>
-    <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="6" t="n">
+    <row r="32" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="6">
         <v>25</v>
       </c>
       <c r="B32" s="6" t="s">
@@ -1319,8 +1285,8 @@
       </c>
       <c r="G32" s="6"/>
     </row>
-    <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="6" t="n">
+    <row r="33" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="6">
         <v>26</v>
       </c>
       <c r="B33" s="6" t="s">
@@ -1340,8 +1306,8 @@
       </c>
       <c r="G33" s="6"/>
     </row>
-    <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="6" t="n">
+    <row r="34" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="6">
         <v>27</v>
       </c>
       <c r="B34" s="6" t="s">
@@ -1359,8 +1325,8 @@
       <c r="F34" s="6"/>
       <c r="G34" s="6"/>
     </row>
-    <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="6" t="n">
+    <row r="35" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="6">
         <v>28</v>
       </c>
       <c r="B35" s="6" t="s">
@@ -1378,8 +1344,8 @@
       <c r="F35" s="6"/>
       <c r="G35" s="6"/>
     </row>
-    <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="6" t="n">
+    <row r="36" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="6">
         <v>29</v>
       </c>
       <c r="B36" s="6" t="s">
@@ -1397,8 +1363,8 @@
       <c r="F36" s="6"/>
       <c r="G36" s="6"/>
     </row>
-    <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="6" t="n">
+    <row r="37" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="6">
         <v>30</v>
       </c>
       <c r="B37" s="6" t="s">
@@ -1416,8 +1382,8 @@
       <c r="F37" s="6"/>
       <c r="G37" s="6"/>
     </row>
-    <row r="38" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="6" t="n">
+    <row r="38" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="6">
         <v>31</v>
       </c>
       <c r="B38" s="6" t="s">
@@ -1435,8 +1401,8 @@
       <c r="F38" s="6"/>
       <c r="G38" s="6"/>
     </row>
-    <row r="39" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="6" t="n">
+    <row r="39" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="6">
         <v>32</v>
       </c>
       <c r="B39" s="6" t="s">
@@ -1454,8 +1420,8 @@
       <c r="F39" s="6"/>
       <c r="G39" s="6"/>
     </row>
-    <row r="40" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="6" t="n">
+    <row r="40" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="6">
         <v>33</v>
       </c>
       <c r="B40" s="6" t="s">
@@ -1475,8 +1441,8 @@
       </c>
       <c r="G40" s="6"/>
     </row>
-    <row r="41" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="6" t="n">
+    <row r="41" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="6">
         <v>34</v>
       </c>
       <c r="B41" s="6" t="s">
@@ -1494,8 +1460,8 @@
       <c r="F41" s="6"/>
       <c r="G41" s="6"/>
     </row>
-    <row r="42" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="6" t="n">
+    <row r="42" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="6">
         <v>35</v>
       </c>
       <c r="B42" s="6" t="s">
@@ -1513,8 +1479,8 @@
       <c r="F42" s="6"/>
       <c r="G42" s="6"/>
     </row>
-    <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="6" t="n">
+    <row r="43" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="6">
         <v>36</v>
       </c>
       <c r="B43" s="6" t="s">
@@ -1532,8 +1498,8 @@
       <c r="F43" s="6"/>
       <c r="G43" s="6"/>
     </row>
-    <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="6" t="n">
+    <row r="44" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="6">
         <v>37</v>
       </c>
       <c r="B44" s="6" t="s">
@@ -1553,8 +1519,8 @@
       </c>
       <c r="G44" s="6"/>
     </row>
-    <row r="45" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="6" t="n">
+    <row r="45" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="6">
         <v>38</v>
       </c>
       <c r="B45" s="6" t="s">
@@ -1572,8 +1538,8 @@
       <c r="F45" s="6"/>
       <c r="G45" s="6"/>
     </row>
-    <row r="46" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="6" t="n">
+    <row r="46" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="6">
         <v>39</v>
       </c>
       <c r="B46" s="6" t="s">
@@ -1591,8 +1557,8 @@
       <c r="F46" s="6"/>
       <c r="G46" s="6"/>
     </row>
-    <row r="47" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="6" t="n">
+    <row r="47" spans="1:7" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="6">
         <v>40</v>
       </c>
       <c r="B47" s="6" t="s">
@@ -1615,28 +1581,23 @@
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <conditionalFormatting sqref="E8:E47">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
       <formula>"Done"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
       <formula>"In Progress"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+    <cfRule type="cellIs" dxfId="0" priority="4" operator="equal">
       <formula>"Not Started"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E8:E47" type="list">
+    <dataValidation type="list" sqref="E8:E47" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Not Started,In Progress,Done"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>